<commit_message>
Update frontend, backend, test suite, and mobile WebView configurations
</commit_message>
<xml_diff>
--- a/tests/test_results_400_passed.xlsx
+++ b/tests/test_results_400_passed.xlsx
@@ -557,7 +557,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated on August 01, 2026 - 09:30:16 | Total Executed: 420 Test Cases</t>
+          <t>Generated on August 05, 2026 - 12:25:38 | Total Executed: 420 Test Cases</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="K5" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="K10" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="K14" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="K16" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="K18" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="K20" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="K24" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="K26" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="K28" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="K29" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="K30" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="K31" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="K32" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="K33" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="K34" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="K35" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="K36" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="K37" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="K38" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="K39" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="K40" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="K41" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="K42" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="K43" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="K44" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3245,7 @@
       </c>
       <c r="K45" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="K46" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3355,7 @@
       </c>
       <c r="K47" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="K48" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="K49" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="K50" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="K51" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3630,7 @@
       </c>
       <c r="K52" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="K53" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="K54" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3795,7 @@
       </c>
       <c r="K55" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="K56" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="K57" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="K58" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4015,7 +4015,7 @@
       </c>
       <c r="K59" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="K60" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="K61" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="K62" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="K63" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="K64" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="K65" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="K66" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="K67" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4510,7 +4510,7 @@
       </c>
       <c r="K68" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="K69" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="K70" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4675,7 @@
       </c>
       <c r="K71" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="K72" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="K73" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       </c>
       <c r="K74" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4895,7 +4895,7 @@
       </c>
       <c r="K75" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="K76" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="K77" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="K78" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="K79" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5170,7 @@
       </c>
       <c r="K80" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="K81" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="K82" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="K83" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5390,7 @@
       </c>
       <c r="K84" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="K85" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,7 @@
       </c>
       <c r="K86" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="K87" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="K88" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="K89" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="K90" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="K91" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="K92" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5885,7 +5885,7 @@
       </c>
       <c r="K93" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="K94" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="K95" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6050,7 +6050,7 @@
       </c>
       <c r="K96" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6105,7 @@
       </c>
       <c r="K97" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="K98" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="K99" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6270,7 +6270,7 @@
       </c>
       <c r="K100" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6325,7 +6325,7 @@
       </c>
       <c r="K101" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="K102" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="K103" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6490,7 +6490,7 @@
       </c>
       <c r="K104" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6545,7 +6545,7 @@
       </c>
       <c r="K105" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="K106" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6655,7 +6655,7 @@
       </c>
       <c r="K107" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6710,7 +6710,7 @@
       </c>
       <c r="K108" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6765,7 +6765,7 @@
       </c>
       <c r="K109" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6820,7 +6820,7 @@
       </c>
       <c r="K110" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6875,7 +6875,7 @@
       </c>
       <c r="K111" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="K112" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="K113" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7040,7 +7040,7 @@
       </c>
       <c r="K114" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="K115" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7150,7 +7150,7 @@
       </c>
       <c r="K116" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="K117" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7260,7 @@
       </c>
       <c r="K118" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7315,7 +7315,7 @@
       </c>
       <c r="K119" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="K120" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7425,7 +7425,7 @@
       </c>
       <c r="K121" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7480,7 +7480,7 @@
       </c>
       <c r="K122" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7535,7 +7535,7 @@
       </c>
       <c r="K123" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="K124" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7645,7 +7645,7 @@
       </c>
       <c r="K125" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7700,7 +7700,7 @@
       </c>
       <c r="K126" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7755,7 @@
       </c>
       <c r="K127" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="K128" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="K129" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7920,7 +7920,7 @@
       </c>
       <c r="K130" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7975,7 @@
       </c>
       <c r="K131" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8030,7 +8030,7 @@
       </c>
       <c r="K132" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8085,7 +8085,7 @@
       </c>
       <c r="K133" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8140,7 +8140,7 @@
       </c>
       <c r="K134" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="K135" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8250,7 +8250,7 @@
       </c>
       <c r="K136" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="K137" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8360,7 +8360,7 @@
       </c>
       <c r="K138" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8415,7 +8415,7 @@
       </c>
       <c r="K139" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="K140" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8525,7 +8525,7 @@
       </c>
       <c r="K141" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8580,7 +8580,7 @@
       </c>
       <c r="K142" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8635,7 +8635,7 @@
       </c>
       <c r="K143" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="K144" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8745,7 +8745,7 @@
       </c>
       <c r="K145" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="K146" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="K147" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8910,7 +8910,7 @@
       </c>
       <c r="K148" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -8965,7 +8965,7 @@
       </c>
       <c r="K149" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9020,7 +9020,7 @@
       </c>
       <c r="K150" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9075,7 +9075,7 @@
       </c>
       <c r="K151" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9130,7 +9130,7 @@
       </c>
       <c r="K152" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="K153" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9240,7 +9240,7 @@
       </c>
       <c r="K154" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9295,7 +9295,7 @@
       </c>
       <c r="K155" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="K156" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="K157" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9460,7 +9460,7 @@
       </c>
       <c r="K158" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9515,7 +9515,7 @@
       </c>
       <c r="K159" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9570,7 +9570,7 @@
       </c>
       <c r="K160" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9625,7 +9625,7 @@
       </c>
       <c r="K161" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9680,7 +9680,7 @@
       </c>
       <c r="K162" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="K163" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9790,7 +9790,7 @@
       </c>
       <c r="K164" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9845,7 +9845,7 @@
       </c>
       <c r="K165" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9900,7 +9900,7 @@
       </c>
       <c r="K166" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -9955,7 +9955,7 @@
       </c>
       <c r="K167" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10010,7 +10010,7 @@
       </c>
       <c r="K168" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10065,7 +10065,7 @@
       </c>
       <c r="K169" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10120,7 +10120,7 @@
       </c>
       <c r="K170" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10175,7 +10175,7 @@
       </c>
       <c r="K171" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10230,7 +10230,7 @@
       </c>
       <c r="K172" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10285,7 +10285,7 @@
       </c>
       <c r="K173" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10340,7 +10340,7 @@
       </c>
       <c r="K174" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10395,7 +10395,7 @@
       </c>
       <c r="K175" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="K176" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="K177" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10560,7 +10560,7 @@
       </c>
       <c r="K178" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10615,7 +10615,7 @@
       </c>
       <c r="K179" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10670,7 +10670,7 @@
       </c>
       <c r="K180" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10725,7 +10725,7 @@
       </c>
       <c r="K181" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10780,7 +10780,7 @@
       </c>
       <c r="K182" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10835,7 +10835,7 @@
       </c>
       <c r="K183" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10890,7 +10890,7 @@
       </c>
       <c r="K184" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -10945,7 +10945,7 @@
       </c>
       <c r="K185" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11000,7 +11000,7 @@
       </c>
       <c r="K186" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11055,7 +11055,7 @@
       </c>
       <c r="K187" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11110,7 +11110,7 @@
       </c>
       <c r="K188" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11165,7 +11165,7 @@
       </c>
       <c r="K189" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11220,7 +11220,7 @@
       </c>
       <c r="K190" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11275,7 +11275,7 @@
       </c>
       <c r="K191" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11330,7 +11330,7 @@
       </c>
       <c r="K192" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11385,7 +11385,7 @@
       </c>
       <c r="K193" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11440,7 +11440,7 @@
       </c>
       <c r="K194" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11495,7 +11495,7 @@
       </c>
       <c r="K195" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11550,7 +11550,7 @@
       </c>
       <c r="K196" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11605,7 +11605,7 @@
       </c>
       <c r="K197" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11660,7 +11660,7 @@
       </c>
       <c r="K198" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11715,7 +11715,7 @@
       </c>
       <c r="K199" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11770,7 +11770,7 @@
       </c>
       <c r="K200" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11825,7 +11825,7 @@
       </c>
       <c r="K201" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11880,7 +11880,7 @@
       </c>
       <c r="K202" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11935,7 +11935,7 @@
       </c>
       <c r="K203" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="K204" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12045,7 +12045,7 @@
       </c>
       <c r="K205" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12100,7 +12100,7 @@
       </c>
       <c r="K206" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12155,7 +12155,7 @@
       </c>
       <c r="K207" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12210,7 +12210,7 @@
       </c>
       <c r="K208" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12265,7 +12265,7 @@
       </c>
       <c r="K209" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12320,7 +12320,7 @@
       </c>
       <c r="K210" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12375,7 +12375,7 @@
       </c>
       <c r="K211" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12430,7 +12430,7 @@
       </c>
       <c r="K212" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12485,7 +12485,7 @@
       </c>
       <c r="K213" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12540,7 +12540,7 @@
       </c>
       <c r="K214" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12595,7 +12595,7 @@
       </c>
       <c r="K215" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12650,7 +12650,7 @@
       </c>
       <c r="K216" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="K217" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12760,7 +12760,7 @@
       </c>
       <c r="K218" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12815,7 @@
       </c>
       <c r="K219" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12870,7 +12870,7 @@
       </c>
       <c r="K220" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12925,7 +12925,7 @@
       </c>
       <c r="K221" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -12980,7 +12980,7 @@
       </c>
       <c r="K222" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13035,7 +13035,7 @@
       </c>
       <c r="K223" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13090,7 +13090,7 @@
       </c>
       <c r="K224" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13145,7 +13145,7 @@
       </c>
       <c r="K225" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13200,7 +13200,7 @@
       </c>
       <c r="K226" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13255,7 +13255,7 @@
       </c>
       <c r="K227" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13310,7 +13310,7 @@
       </c>
       <c r="K228" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13365,7 +13365,7 @@
       </c>
       <c r="K229" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13420,7 +13420,7 @@
       </c>
       <c r="K230" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13475,7 +13475,7 @@
       </c>
       <c r="K231" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13530,7 +13530,7 @@
       </c>
       <c r="K232" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13585,7 +13585,7 @@
       </c>
       <c r="K233" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13640,7 +13640,7 @@
       </c>
       <c r="K234" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13695,7 +13695,7 @@
       </c>
       <c r="K235" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13750,7 +13750,7 @@
       </c>
       <c r="K236" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13805,7 +13805,7 @@
       </c>
       <c r="K237" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13860,7 +13860,7 @@
       </c>
       <c r="K238" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13915,7 +13915,7 @@
       </c>
       <c r="K239" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -13970,7 +13970,7 @@
       </c>
       <c r="K240" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14025,7 +14025,7 @@
       </c>
       <c r="K241" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14080,7 +14080,7 @@
       </c>
       <c r="K242" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14135,7 +14135,7 @@
       </c>
       <c r="K243" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14190,7 +14190,7 @@
       </c>
       <c r="K244" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14245,7 +14245,7 @@
       </c>
       <c r="K245" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14300,7 +14300,7 @@
       </c>
       <c r="K246" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14355,7 +14355,7 @@
       </c>
       <c r="K247" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14410,7 +14410,7 @@
       </c>
       <c r="K248" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14465,7 +14465,7 @@
       </c>
       <c r="K249" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14520,7 +14520,7 @@
       </c>
       <c r="K250" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14575,7 +14575,7 @@
       </c>
       <c r="K251" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14630,7 +14630,7 @@
       </c>
       <c r="K252" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14685,7 +14685,7 @@
       </c>
       <c r="K253" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14740,7 +14740,7 @@
       </c>
       <c r="K254" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14795,7 +14795,7 @@
       </c>
       <c r="K255" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14850,7 +14850,7 @@
       </c>
       <c r="K256" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14905,7 +14905,7 @@
       </c>
       <c r="K257" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -14960,7 +14960,7 @@
       </c>
       <c r="K258" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15015,7 +15015,7 @@
       </c>
       <c r="K259" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15070,7 +15070,7 @@
       </c>
       <c r="K260" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15125,7 +15125,7 @@
       </c>
       <c r="K261" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15180,7 +15180,7 @@
       </c>
       <c r="K262" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15235,7 +15235,7 @@
       </c>
       <c r="K263" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15290,7 +15290,7 @@
       </c>
       <c r="K264" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15345,7 +15345,7 @@
       </c>
       <c r="K265" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15400,7 +15400,7 @@
       </c>
       <c r="K266" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15455,7 +15455,7 @@
       </c>
       <c r="K267" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15510,7 +15510,7 @@
       </c>
       <c r="K268" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="K269" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15620,7 +15620,7 @@
       </c>
       <c r="K270" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15675,7 +15675,7 @@
       </c>
       <c r="K271" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15730,7 +15730,7 @@
       </c>
       <c r="K272" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15785,7 +15785,7 @@
       </c>
       <c r="K273" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="K274" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15895,7 +15895,7 @@
       </c>
       <c r="K275" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -15950,7 +15950,7 @@
       </c>
       <c r="K276" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16005,7 +16005,7 @@
       </c>
       <c r="K277" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="K278" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16115,7 +16115,7 @@
       </c>
       <c r="K279" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16170,7 +16170,7 @@
       </c>
       <c r="K280" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16225,7 +16225,7 @@
       </c>
       <c r="K281" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16280,7 +16280,7 @@
       </c>
       <c r="K282" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16335,7 +16335,7 @@
       </c>
       <c r="K283" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16390,7 +16390,7 @@
       </c>
       <c r="K284" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16445,7 +16445,7 @@
       </c>
       <c r="K285" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16500,7 +16500,7 @@
       </c>
       <c r="K286" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16555,7 +16555,7 @@
       </c>
       <c r="K287" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16610,7 +16610,7 @@
       </c>
       <c r="K288" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="K289" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16720,7 +16720,7 @@
       </c>
       <c r="K290" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16775,7 +16775,7 @@
       </c>
       <c r="K291" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16830,7 +16830,7 @@
       </c>
       <c r="K292" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16885,7 +16885,7 @@
       </c>
       <c r="K293" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16940,7 +16940,7 @@
       </c>
       <c r="K294" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -16995,7 +16995,7 @@
       </c>
       <c r="K295" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17050,7 +17050,7 @@
       </c>
       <c r="K296" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17105,7 +17105,7 @@
       </c>
       <c r="K297" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="K298" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17215,7 +17215,7 @@
       </c>
       <c r="K299" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17270,7 +17270,7 @@
       </c>
       <c r="K300" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17325,7 +17325,7 @@
       </c>
       <c r="K301" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17380,7 +17380,7 @@
       </c>
       <c r="K302" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17435,7 +17435,7 @@
       </c>
       <c r="K303" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17490,7 +17490,7 @@
       </c>
       <c r="K304" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17545,7 +17545,7 @@
       </c>
       <c r="K305" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17600,7 +17600,7 @@
       </c>
       <c r="K306" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17655,7 +17655,7 @@
       </c>
       <c r="K307" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17710,7 +17710,7 @@
       </c>
       <c r="K308" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17765,7 +17765,7 @@
       </c>
       <c r="K309" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17820,7 +17820,7 @@
       </c>
       <c r="K310" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17875,7 +17875,7 @@
       </c>
       <c r="K311" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17930,7 +17930,7 @@
       </c>
       <c r="K312" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -17985,7 +17985,7 @@
       </c>
       <c r="K313" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18040,7 +18040,7 @@
       </c>
       <c r="K314" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18095,7 +18095,7 @@
       </c>
       <c r="K315" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18150,7 +18150,7 @@
       </c>
       <c r="K316" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18205,7 +18205,7 @@
       </c>
       <c r="K317" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18260,7 +18260,7 @@
       </c>
       <c r="K318" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18315,7 +18315,7 @@
       </c>
       <c r="K319" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18370,7 +18370,7 @@
       </c>
       <c r="K320" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18425,7 +18425,7 @@
       </c>
       <c r="K321" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18480,7 +18480,7 @@
       </c>
       <c r="K322" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18535,7 +18535,7 @@
       </c>
       <c r="K323" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18590,7 +18590,7 @@
       </c>
       <c r="K324" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18645,7 +18645,7 @@
       </c>
       <c r="K325" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18700,7 +18700,7 @@
       </c>
       <c r="K326" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18755,7 +18755,7 @@
       </c>
       <c r="K327" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18810,7 +18810,7 @@
       </c>
       <c r="K328" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18865,7 +18865,7 @@
       </c>
       <c r="K329" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18920,7 +18920,7 @@
       </c>
       <c r="K330" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -18975,7 +18975,7 @@
       </c>
       <c r="K331" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19030,7 +19030,7 @@
       </c>
       <c r="K332" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19085,7 +19085,7 @@
       </c>
       <c r="K333" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19140,7 +19140,7 @@
       </c>
       <c r="K334" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19195,7 +19195,7 @@
       </c>
       <c r="K335" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19250,7 +19250,7 @@
       </c>
       <c r="K336" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19305,7 +19305,7 @@
       </c>
       <c r="K337" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19360,7 +19360,7 @@
       </c>
       <c r="K338" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19415,7 +19415,7 @@
       </c>
       <c r="K339" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19470,7 +19470,7 @@
       </c>
       <c r="K340" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19525,7 +19525,7 @@
       </c>
       <c r="K341" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19580,7 +19580,7 @@
       </c>
       <c r="K342" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19635,7 +19635,7 @@
       </c>
       <c r="K343" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19690,7 +19690,7 @@
       </c>
       <c r="K344" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19745,7 +19745,7 @@
       </c>
       <c r="K345" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19800,7 +19800,7 @@
       </c>
       <c r="K346" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19855,7 +19855,7 @@
       </c>
       <c r="K347" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19910,7 +19910,7 @@
       </c>
       <c r="K348" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -19965,7 +19965,7 @@
       </c>
       <c r="K349" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20020,7 +20020,7 @@
       </c>
       <c r="K350" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20075,7 +20075,7 @@
       </c>
       <c r="K351" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20130,7 +20130,7 @@
       </c>
       <c r="K352" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20185,7 +20185,7 @@
       </c>
       <c r="K353" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20240,7 +20240,7 @@
       </c>
       <c r="K354" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20295,7 +20295,7 @@
       </c>
       <c r="K355" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20350,7 +20350,7 @@
       </c>
       <c r="K356" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20405,7 +20405,7 @@
       </c>
       <c r="K357" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20460,7 +20460,7 @@
       </c>
       <c r="K358" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20515,7 +20515,7 @@
       </c>
       <c r="K359" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20570,7 +20570,7 @@
       </c>
       <c r="K360" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20625,7 +20625,7 @@
       </c>
       <c r="K361" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20680,7 +20680,7 @@
       </c>
       <c r="K362" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20735,7 +20735,7 @@
       </c>
       <c r="K363" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20790,7 +20790,7 @@
       </c>
       <c r="K364" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20845,7 +20845,7 @@
       </c>
       <c r="K365" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20900,7 +20900,7 @@
       </c>
       <c r="K366" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -20955,7 +20955,7 @@
       </c>
       <c r="K367" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21010,7 +21010,7 @@
       </c>
       <c r="K368" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21065,7 +21065,7 @@
       </c>
       <c r="K369" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21120,7 +21120,7 @@
       </c>
       <c r="K370" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21175,7 +21175,7 @@
       </c>
       <c r="K371" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21230,7 +21230,7 @@
       </c>
       <c r="K372" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21285,7 +21285,7 @@
       </c>
       <c r="K373" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21340,7 +21340,7 @@
       </c>
       <c r="K374" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21395,7 +21395,7 @@
       </c>
       <c r="K375" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       </c>
       <c r="K376" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21505,7 +21505,7 @@
       </c>
       <c r="K377" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21560,7 +21560,7 @@
       </c>
       <c r="K378" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21615,7 +21615,7 @@
       </c>
       <c r="K379" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21670,7 +21670,7 @@
       </c>
       <c r="K380" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21725,7 +21725,7 @@
       </c>
       <c r="K381" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21780,7 +21780,7 @@
       </c>
       <c r="K382" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21835,7 +21835,7 @@
       </c>
       <c r="K383" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21890,7 +21890,7 @@
       </c>
       <c r="K384" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -21945,7 +21945,7 @@
       </c>
       <c r="K385" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22000,7 +22000,7 @@
       </c>
       <c r="K386" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22055,7 +22055,7 @@
       </c>
       <c r="K387" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22110,7 +22110,7 @@
       </c>
       <c r="K388" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22165,7 +22165,7 @@
       </c>
       <c r="K389" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22220,7 +22220,7 @@
       </c>
       <c r="K390" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22275,7 +22275,7 @@
       </c>
       <c r="K391" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22330,7 +22330,7 @@
       </c>
       <c r="K392" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22385,7 +22385,7 @@
       </c>
       <c r="K393" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22440,7 +22440,7 @@
       </c>
       <c r="K394" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22495,7 +22495,7 @@
       </c>
       <c r="K395" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22550,7 +22550,7 @@
       </c>
       <c r="K396" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22605,7 +22605,7 @@
       </c>
       <c r="K397" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22660,7 +22660,7 @@
       </c>
       <c r="K398" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22715,7 +22715,7 @@
       </c>
       <c r="K399" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22770,7 +22770,7 @@
       </c>
       <c r="K400" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22825,7 +22825,7 @@
       </c>
       <c r="K401" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22880,7 +22880,7 @@
       </c>
       <c r="K402" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22935,7 +22935,7 @@
       </c>
       <c r="K403" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -22990,7 +22990,7 @@
       </c>
       <c r="K404" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23045,7 +23045,7 @@
       </c>
       <c r="K405" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23100,7 +23100,7 @@
       </c>
       <c r="K406" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23155,7 +23155,7 @@
       </c>
       <c r="K407" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23210,7 +23210,7 @@
       </c>
       <c r="K408" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23265,7 +23265,7 @@
       </c>
       <c r="K409" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23320,7 +23320,7 @@
       </c>
       <c r="K410" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23375,7 +23375,7 @@
       </c>
       <c r="K411" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23430,7 +23430,7 @@
       </c>
       <c r="K412" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23485,7 +23485,7 @@
       </c>
       <c r="K413" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23540,7 +23540,7 @@
       </c>
       <c r="K414" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23595,7 +23595,7 @@
       </c>
       <c r="K415" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="K416" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23705,7 +23705,7 @@
       </c>
       <c r="K417" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23760,7 +23760,7 @@
       </c>
       <c r="K418" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23815,7 +23815,7 @@
       </c>
       <c r="K419" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23870,7 +23870,7 @@
       </c>
       <c r="K420" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>
@@ -23925,7 +23925,7 @@
       </c>
       <c r="K421" s="9" t="inlineStr">
         <is>
-          <t>2026-08-01 09:30:16</t>
+          <t>2026-08-05 12:25:38</t>
         </is>
       </c>
     </row>

</xml_diff>